<commit_message>
Retire l'onglet VO du gabarit Excel exporté
</commit_message>
<xml_diff>
--- a/public/templates/trame_renta_template.xlsx
+++ b/public/templates/trame_renta_template.xlsx
@@ -10,11 +10,10 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FABA9B8-25AB-A14F-B1A0-6D7AB2F044B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RENTA VN" sheetId="1" r:id="rId1"/>
-    <sheet name="RENTA VO" sheetId="2" r:id="rId2"/>
     <sheet name="DONNEES" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
@@ -74,58 +73,6 @@
             <family val="2"/>
           </rPr>
           <t>Coût moyen par transporteur : 350€ HT</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Unknown Author</author>
-  </authors>
-  <commentList>
-    <comment ref="B2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t>Légende :
-- Fond rose pâle = cellule de saisie
-- Texte rose foncé = valeur calculée automatiquement
-- Feuille protégée : seules les cellules de saisie sont modifiables</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve"> Garantie - 4ans &amp; - 40 000 Km = 242€
- Garantie - 8ans &amp; - 80 000 Km = 363€
- Garantie - 12ans &amp; - 120 000 Km = 581€
- Garantie - 16 ans &amp; - 160 000 Km = 472€</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t>Coût moyen par transporteur : 350 € HT</t>
         </r>
       </text>
     </comment>
@@ -3609,1705 +3556,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:M81"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="2.5" style="15" customWidth="1"/>
-    <col min="2" max="2" width="30" style="16" customWidth="1"/>
-    <col min="3" max="5" width="13" style="16" customWidth="1"/>
-    <col min="6" max="6" width="2.5" style="16" customWidth="1"/>
-    <col min="7" max="7" width="34" style="16" customWidth="1"/>
-    <col min="8" max="8" width="12" style="16" customWidth="1"/>
-    <col min="9" max="11" width="13" style="16" customWidth="1"/>
-    <col min="12" max="12" width="11" style="15" customWidth="1"/>
-    <col min="13" max="13" width="26.6640625" style="15" customWidth="1"/>
-    <col min="14" max="16384" width="11.5" style="16"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="17"/>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-    </row>
-    <row r="2" spans="1:12" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17"/>
-      <c r="B2" s="115" t="s">
-        <v>66</v>
-      </c>
-      <c r="C2" s="115"/>
-      <c r="D2" s="115"/>
-      <c r="E2" s="115"/>
-      <c r="F2" s="115"/>
-      <c r="G2" s="115"/>
-      <c r="H2" s="116" t="str">
-        <f>IF(G8="Moins de 360 jours",(I8+J46-J30)/50,(I8+J46)/50)&amp; " Heures DANS L'ATELIER (Prépa, Mise en main)"</f>
-        <v>6 Heures DANS L'ATELIER (Prépa, Mise en main)</v>
-      </c>
-      <c r="I2" s="116"/>
-      <c r="J2" s="116"/>
-      <c r="K2" s="116"/>
-      <c r="L2" s="116"/>
-    </row>
-    <row r="3" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-    </row>
-    <row r="4" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="17"/>
-      <c r="B4" s="117" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="117"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="117"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="118" t="s">
-        <v>2</v>
-      </c>
-      <c r="H4" s="118"/>
-      <c r="I4" s="119" t="s">
-        <v>67</v>
-      </c>
-      <c r="J4" s="119"/>
-      <c r="K4" s="119"/>
-      <c r="L4" s="119"/>
-    </row>
-    <row r="5" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="17"/>
-      <c r="B5" s="63" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="120"/>
-      <c r="D5" s="120"/>
-      <c r="E5" s="120"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="121" t="s">
-        <v>5</v>
-      </c>
-      <c r="H5" s="121"/>
-      <c r="I5" s="122">
-        <f>IF(G5="Camping car",235,(IF(G5="CARAVANE",120,0)))</f>
-        <v>235</v>
-      </c>
-      <c r="J5" s="122"/>
-      <c r="K5" s="123" t="str">
-        <f>IF(G5="Camping car","790 € TTC CLIENT",(IF(G5="CARAVANE","380 € TTC CLIENT","PAS DE FORFAIT ADMIN")))</f>
-        <v>790 € TTC CLIENT</v>
-      </c>
-      <c r="L5" s="123"/>
-    </row>
-    <row r="6" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="17"/>
-      <c r="B6" s="63" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="120"/>
-      <c r="D6" s="120"/>
-      <c r="E6" s="120"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="121"/>
-      <c r="H6" s="121"/>
-      <c r="I6" s="122"/>
-      <c r="J6" s="122"/>
-      <c r="K6" s="123"/>
-      <c r="L6" s="123"/>
-    </row>
-    <row r="7" spans="1:12" s="15" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="17"/>
-      <c r="B7" s="63" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="124"/>
-      <c r="D7" s="124"/>
-      <c r="E7" s="124"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="118" t="s">
-        <v>68</v>
-      </c>
-      <c r="H7" s="118"/>
-      <c r="I7" s="119" t="s">
-        <v>69</v>
-      </c>
-      <c r="J7" s="119"/>
-      <c r="K7" s="119"/>
-      <c r="L7" s="119"/>
-    </row>
-    <row r="8" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="17"/>
-      <c r="B8" s="63" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="124"/>
-      <c r="D8" s="124"/>
-      <c r="E8" s="124"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="125" t="s">
-        <v>70</v>
-      </c>
-      <c r="H8" s="125"/>
-      <c r="I8" s="122">
-        <f>IF(G5="Camping car",300,(IF(G5="CARAVANE",250,0)))</f>
-        <v>300</v>
-      </c>
-      <c r="J8" s="122"/>
-      <c r="K8" s="123" t="str">
-        <f>IF(G5="Camping car","6 Heures",(IF(G5="CARAVANE","5 Heures","0H")))</f>
-        <v>6 Heures</v>
-      </c>
-      <c r="L8" s="123"/>
-    </row>
-    <row r="9" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="17"/>
-      <c r="B9" s="65" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="126">
-        <f>IF(E36=0,(E35*8%),(E35*10%+E41*0.3%))</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="126"/>
-      <c r="E9" s="126"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="125"/>
-      <c r="H9" s="125"/>
-      <c r="I9" s="122"/>
-      <c r="J9" s="122"/>
-      <c r="K9" s="123"/>
-      <c r="L9" s="123"/>
-    </row>
-    <row r="10" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="17"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="19"/>
-    </row>
-    <row r="11" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="17"/>
-      <c r="B11" s="117" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="117"/>
-      <c r="D11" s="117"/>
-      <c r="E11" s="117"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="127" t="s">
-        <v>71</v>
-      </c>
-      <c r="H11" s="127"/>
-      <c r="I11" s="127"/>
-      <c r="J11" s="127"/>
-      <c r="K11" s="127"/>
-      <c r="L11" s="127"/>
-    </row>
-    <row r="12" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="17"/>
-      <c r="B12" s="63" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="124"/>
-      <c r="D12" s="124"/>
-      <c r="E12" s="124"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="128" t="s">
-        <v>72</v>
-      </c>
-      <c r="H12" s="128"/>
-      <c r="I12" s="128"/>
-      <c r="J12" s="67" t="s">
-        <v>73</v>
-      </c>
-      <c r="K12" s="129" t="s">
-        <v>74</v>
-      </c>
-      <c r="L12" s="129"/>
-    </row>
-    <row r="13" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="17"/>
-      <c r="B13" s="63" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="124"/>
-      <c r="D13" s="124"/>
-      <c r="E13" s="124"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="130" t="s">
-        <v>75</v>
-      </c>
-      <c r="H13" s="130"/>
-      <c r="I13" s="130"/>
-      <c r="J13" s="68" t="s">
-        <v>52</v>
-      </c>
-      <c r="K13" s="131">
-        <f>IF(J13="OUI",150,0)</f>
-        <v>0</v>
-      </c>
-      <c r="L13" s="131"/>
-    </row>
-    <row r="14" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="17"/>
-      <c r="B14" s="63" t="s">
-        <v>76</v>
-      </c>
-      <c r="C14" s="120"/>
-      <c r="D14" s="120"/>
-      <c r="E14" s="120"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="130" t="s">
-        <v>77</v>
-      </c>
-      <c r="H14" s="130"/>
-      <c r="I14" s="130"/>
-      <c r="J14" s="68" t="s">
-        <v>52</v>
-      </c>
-      <c r="K14" s="131">
-        <f>IF(J14="OUI",300,0)</f>
-        <v>0</v>
-      </c>
-      <c r="L14" s="131"/>
-    </row>
-    <row r="15" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="17"/>
-      <c r="B15" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C15" s="124"/>
-      <c r="D15" s="124"/>
-      <c r="E15" s="124"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="130" t="s">
-        <v>79</v>
-      </c>
-      <c r="H15" s="130"/>
-      <c r="I15" s="130"/>
-      <c r="J15" s="68" t="s">
-        <v>52</v>
-      </c>
-      <c r="K15" s="131">
-        <f>IF(J15="OUI",600,0)</f>
-        <v>0</v>
-      </c>
-      <c r="L15" s="131"/>
-    </row>
-    <row r="16" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="17"/>
-      <c r="B16" s="63" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="120"/>
-      <c r="D16" s="120"/>
-      <c r="E16" s="120"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="130" t="s">
-        <v>80</v>
-      </c>
-      <c r="H16" s="130"/>
-      <c r="I16" s="130"/>
-      <c r="J16" s="68" t="s">
-        <v>52</v>
-      </c>
-      <c r="K16" s="131">
-        <f>IF(J16="OUI",850,0)</f>
-        <v>0</v>
-      </c>
-      <c r="L16" s="131"/>
-    </row>
-    <row r="17" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="17"/>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="130" t="s">
-        <v>81</v>
-      </c>
-      <c r="H17" s="130"/>
-      <c r="I17" s="130"/>
-      <c r="J17" s="68" t="s">
-        <v>52</v>
-      </c>
-      <c r="K17" s="131">
-        <f>IF(J17="NON",0,IF(J17="OUI, 1 en 15""",400,IF(J17="OUI, 2 en 15""",800,IF(J17="OUI, 1 en 16""",500,1000))))</f>
-        <v>0</v>
-      </c>
-      <c r="L17" s="131"/>
-    </row>
-    <row r="18" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="17"/>
-      <c r="B18" s="148" t="s">
-        <v>25</v>
-      </c>
-      <c r="C18" s="148"/>
-      <c r="D18" s="148"/>
-      <c r="E18" s="148"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="130" t="s">
-        <v>82</v>
-      </c>
-      <c r="H18" s="130"/>
-      <c r="I18" s="130"/>
-      <c r="J18" s="68" t="s">
-        <v>52</v>
-      </c>
-      <c r="K18" s="131">
-        <f>IF(J18="OUI",70,0)</f>
-        <v>0</v>
-      </c>
-      <c r="L18" s="131"/>
-    </row>
-    <row r="19" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="17"/>
-      <c r="B19" s="132" t="s">
-        <v>83</v>
-      </c>
-      <c r="C19" s="132"/>
-      <c r="D19" s="132"/>
-      <c r="E19" s="70"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="130" t="s">
-        <v>84</v>
-      </c>
-      <c r="H19" s="130"/>
-      <c r="I19" s="130"/>
-      <c r="J19" s="68" t="s">
-        <v>52</v>
-      </c>
-      <c r="K19" s="131">
-        <f>IF(J19="OUI, VL",80,(IF(J19="OUI, PL",120,0)))</f>
-        <v>0</v>
-      </c>
-      <c r="L19" s="131"/>
-    </row>
-    <row r="20" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="17"/>
-      <c r="B20" s="132" t="s">
-        <v>28</v>
-      </c>
-      <c r="C20" s="132"/>
-      <c r="D20" s="132"/>
-      <c r="E20" s="70"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="130" t="s">
-        <v>85</v>
-      </c>
-      <c r="H20" s="130"/>
-      <c r="I20" s="130"/>
-      <c r="J20" s="68" t="s">
-        <v>52</v>
-      </c>
-      <c r="K20" s="131">
-        <f>IF(J20="OUI",50,0)</f>
-        <v>0</v>
-      </c>
-      <c r="L20" s="131"/>
-    </row>
-    <row r="21" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="17"/>
-      <c r="B21" s="132" t="s">
-        <v>86</v>
-      </c>
-      <c r="C21" s="132"/>
-      <c r="D21" s="132"/>
-      <c r="E21" s="70"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="130" t="s">
-        <v>87</v>
-      </c>
-      <c r="H21" s="130"/>
-      <c r="I21" s="130"/>
-      <c r="J21" s="68" t="s">
-        <v>52</v>
-      </c>
-      <c r="K21" s="133" t="s">
-        <v>88</v>
-      </c>
-      <c r="L21" s="133"/>
-    </row>
-    <row r="22" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="17"/>
-      <c r="B22" s="134" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" s="134"/>
-      <c r="D22" s="134"/>
-      <c r="E22" s="71"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="130" t="s">
-        <v>89</v>
-      </c>
-      <c r="H22" s="130"/>
-      <c r="I22" s="130"/>
-      <c r="J22" s="68" t="s">
-        <v>52</v>
-      </c>
-      <c r="K22" s="133" t="s">
-        <v>88</v>
-      </c>
-      <c r="L22" s="133"/>
-    </row>
-    <row r="23" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="17"/>
-      <c r="B23" s="134" t="s">
-        <v>90</v>
-      </c>
-      <c r="C23" s="134"/>
-      <c r="D23" s="134"/>
-      <c r="E23" s="66">
-        <f>E27-E19</f>
-        <v>0</v>
-      </c>
-      <c r="F23" s="19"/>
-      <c r="G23" s="130" t="s">
-        <v>89</v>
-      </c>
-      <c r="H23" s="130"/>
-      <c r="I23" s="130"/>
-      <c r="J23" s="68" t="s">
-        <v>52</v>
-      </c>
-      <c r="K23" s="133" t="s">
-        <v>88</v>
-      </c>
-      <c r="L23" s="133"/>
-    </row>
-    <row r="24" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="17"/>
-      <c r="B24" s="135" t="s">
-        <v>91</v>
-      </c>
-      <c r="C24" s="135"/>
-      <c r="D24" s="135"/>
-      <c r="E24" s="69">
-        <f>IF(E23&gt;0,(E23/1.2)*0.2,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F24" s="19"/>
-      <c r="G24" s="136" t="s">
-        <v>34</v>
-      </c>
-      <c r="H24" s="136"/>
-      <c r="I24" s="136"/>
-      <c r="J24" s="73"/>
-      <c r="K24" s="137">
-        <f>SUM(K13:L23)</f>
-        <v>0</v>
-      </c>
-      <c r="L24" s="137"/>
-    </row>
-    <row r="25" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="17"/>
-      <c r="B25" s="135" t="s">
-        <v>92</v>
-      </c>
-      <c r="C25" s="135"/>
-      <c r="D25" s="135"/>
-      <c r="E25" s="58"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
-      <c r="J25" s="19"/>
-      <c r="K25" s="19"/>
-      <c r="L25" s="19"/>
-    </row>
-    <row r="26" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="17"/>
-      <c r="B26" s="135" t="s">
-        <v>93</v>
-      </c>
-      <c r="C26" s="135"/>
-      <c r="D26" s="135"/>
-      <c r="E26" s="66">
-        <f>E25+K46</f>
-        <v>0</v>
-      </c>
-      <c r="F26" s="19"/>
-      <c r="G26" s="138" t="s">
-        <v>36</v>
-      </c>
-      <c r="H26" s="138"/>
-      <c r="I26" s="138"/>
-      <c r="J26" s="138"/>
-      <c r="K26" s="138"/>
-      <c r="L26" s="138"/>
-    </row>
-    <row r="27" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="17"/>
-      <c r="B27" s="132" t="s">
-        <v>32</v>
-      </c>
-      <c r="C27" s="132"/>
-      <c r="D27" s="132"/>
-      <c r="E27" s="70"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="139" t="s">
-        <v>94</v>
-      </c>
-      <c r="H27" s="139"/>
-      <c r="I27" s="75" t="s">
-        <v>39</v>
-      </c>
-      <c r="J27" s="75" t="s">
-        <v>95</v>
-      </c>
-      <c r="K27" s="75" t="s">
-        <v>18</v>
-      </c>
-      <c r="L27" s="75" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="17"/>
-      <c r="B28" s="134" t="s">
-        <v>33</v>
-      </c>
-      <c r="C28" s="134"/>
-      <c r="D28" s="76">
-        <f>IFERROR(IF(E28=0,0,E28/E26),0)</f>
-        <v>0</v>
-      </c>
-      <c r="E28" s="66">
-        <f>E26-E27</f>
-        <v>0</v>
-      </c>
-      <c r="F28" s="19"/>
-      <c r="G28" s="140" t="s">
-        <v>42</v>
-      </c>
-      <c r="H28" s="140"/>
-      <c r="I28" s="69">
-        <f>IF(G5="CARAVANE",0,300)</f>
-        <v>300</v>
-      </c>
-      <c r="J28" s="46"/>
-      <c r="K28" s="46"/>
-      <c r="L28" s="47" t="str">
-        <f t="shared" ref="L28:L45" si="0">J28/50&amp;" H"</f>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="17"/>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="77"/>
-      <c r="E29" s="78"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="140" t="s">
-        <v>46</v>
-      </c>
-      <c r="H29" s="140"/>
-      <c r="I29" s="70">
-        <v>250</v>
-      </c>
-      <c r="J29" s="79"/>
-      <c r="K29" s="79"/>
-      <c r="L29" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="17"/>
-      <c r="B30" s="141" t="s">
-        <v>35</v>
-      </c>
-      <c r="C30" s="141"/>
-      <c r="D30" s="141"/>
-      <c r="E30" s="80">
-        <f>SUM(E31:E32)</f>
-        <v>5000</v>
-      </c>
-      <c r="F30" s="19"/>
-      <c r="G30" s="142" t="str">
-        <f>IF(OR(G5="PROTO A MARCHAND (VDL &gt; 2014)",G5="PROTO A MARCHAND (VDL &lt; 2014)"),"PAS DE SUPPLEMENT",(IF(G8="Moins de 360 jours","Moins de 360 jours : + 3H MO = SURPRISE","Plus de 361 jours : +3H MO et changement batterie cellule si CC")))</f>
-        <v>Moins de 360 jours : + 3H MO = SURPRISE</v>
-      </c>
-      <c r="H30" s="142"/>
-      <c r="I30" s="69">
-        <f>IF(OR(G5="PROTO A MARCHAND (VDL &gt; 2014)",G5="PROTO A MARCHAND (VDL &lt; 2014)"),0,(IF(G5="CARAVANE",0,(IF(G8="Moins de 360 jours",0,192)))))</f>
-        <v>0</v>
-      </c>
-      <c r="J30" s="69">
-        <f>IF(OR(G5="PROTO A MARCHAND (VDL &gt; 2014)",G5="PROTO A MARCHAND (VDL &lt; 2014)"),0,(IF(G5="CARAVANE",150,(IF(G8="Moins de 360 jours",150,200)))))</f>
-        <v>150</v>
-      </c>
-      <c r="K30" s="79"/>
-      <c r="L30" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>3 H</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="17"/>
-      <c r="B31" s="135" t="s">
-        <v>37</v>
-      </c>
-      <c r="C31" s="135"/>
-      <c r="D31" s="135"/>
-      <c r="E31" s="81">
-        <f>IF(AND(G5="CAMPING CAR",G8="Moins de 360 jours"),5000,(IF(AND(G5="CAMPING CAR",G8="Entre 361 et 700 jours"),3500,(IF(AND(G5="CARAVANE",G8="Moins de 360 jours"),2500,(IF(AND(G5="CARAVANE",G8="Entre 361 et 700 jours"),1500,(IF(G8="Plus de 701 jours","DESTOCKAGE",(IF(AND(G5="PROTO A MARCHAND (VDL &gt; 2014)",G8="Moins de 360 jours"),5000,(IF(AND(G5="PROTO A MARCHAND (VDL &gt; 2014)",G8="Entre 361 et 700 jours"),3500,(IF(AND(G5="PROTO A MARCHAND (VDL &lt; 2014)",G8="Moins de 360 jours"),3500,(IF(AND(G5="PROTO A MARCHAND (VDL &lt; 2014)",G8="Entre 361 et 700 jours"),3500)))))))))))))))))</f>
-        <v>5000</v>
-      </c>
-      <c r="F31" s="19"/>
-      <c r="G31" s="108"/>
-      <c r="H31" s="108"/>
-      <c r="I31" s="53"/>
-      <c r="J31" s="53"/>
-      <c r="K31" s="53"/>
-      <c r="L31" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="17"/>
-      <c r="B32" s="135" t="s">
-        <v>41</v>
-      </c>
-      <c r="C32" s="135"/>
-      <c r="D32" s="135"/>
-      <c r="E32" s="81">
-        <f>IF(G5="PROTO A MARCHAND (VDL &lt; 2014)",0,E26*0.3*0.06)</f>
-        <v>0</v>
-      </c>
-      <c r="F32" s="19"/>
-      <c r="G32" s="108"/>
-      <c r="H32" s="108"/>
-      <c r="I32" s="53"/>
-      <c r="J32" s="53"/>
-      <c r="K32" s="53"/>
-      <c r="L32" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="17"/>
-      <c r="B33" s="26"/>
-      <c r="C33" s="26"/>
-      <c r="D33" s="82"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="143"/>
-      <c r="H33" s="143"/>
-      <c r="I33" s="83"/>
-      <c r="J33" s="83"/>
-      <c r="K33" s="83"/>
-      <c r="L33" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="17"/>
-      <c r="B34" s="144" t="s">
-        <v>43</v>
-      </c>
-      <c r="C34" s="144"/>
-      <c r="D34" s="144"/>
-      <c r="E34" s="84">
-        <f>SUM(E35:E36)</f>
-        <v>0</v>
-      </c>
-      <c r="F34" s="19"/>
-      <c r="G34" s="143"/>
-      <c r="H34" s="143"/>
-      <c r="I34" s="83"/>
-      <c r="J34" s="83"/>
-      <c r="K34" s="83"/>
-      <c r="L34" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="17"/>
-      <c r="B35" s="132" t="s">
-        <v>37</v>
-      </c>
-      <c r="C35" s="132"/>
-      <c r="D35" s="132"/>
-      <c r="E35" s="85">
-        <f>IF(E19&gt;0,(E23-E20-E21-E22-E24-I5-I8-K24-I46-J46),0)</f>
-        <v>0</v>
-      </c>
-      <c r="F35" s="19"/>
-      <c r="G35" s="143"/>
-      <c r="H35" s="143"/>
-      <c r="I35" s="83"/>
-      <c r="J35" s="83"/>
-      <c r="K35" s="83"/>
-      <c r="L35" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="17"/>
-      <c r="B36" s="132" t="s">
-        <v>41</v>
-      </c>
-      <c r="C36" s="132"/>
-      <c r="D36" s="132"/>
-      <c r="E36" s="85">
-        <f>E41*0.06</f>
-        <v>0</v>
-      </c>
-      <c r="F36" s="19"/>
-      <c r="G36" s="143"/>
-      <c r="H36" s="143"/>
-      <c r="I36" s="86"/>
-      <c r="J36" s="83"/>
-      <c r="K36" s="83"/>
-      <c r="L36" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="17"/>
-      <c r="B37" s="19"/>
-      <c r="C37" s="19"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="19"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="143"/>
-      <c r="H37" s="143"/>
-      <c r="I37" s="53"/>
-      <c r="J37" s="53"/>
-      <c r="K37" s="53"/>
-      <c r="L37" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="17"/>
-      <c r="B38" s="117" t="s">
-        <v>47</v>
-      </c>
-      <c r="C38" s="117"/>
-      <c r="D38" s="117"/>
-      <c r="E38" s="117"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="143"/>
-      <c r="H38" s="143"/>
-      <c r="I38" s="53"/>
-      <c r="J38" s="53"/>
-      <c r="K38" s="53"/>
-      <c r="L38" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="17"/>
-      <c r="B39" s="135" t="s">
-        <v>47</v>
-      </c>
-      <c r="C39" s="135"/>
-      <c r="D39" s="135"/>
-      <c r="E39" s="87"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="143"/>
-      <c r="H39" s="143"/>
-      <c r="I39" s="53"/>
-      <c r="J39" s="53"/>
-      <c r="K39" s="53"/>
-      <c r="L39" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="17"/>
-      <c r="B40" s="135" t="s">
-        <v>49</v>
-      </c>
-      <c r="C40" s="135"/>
-      <c r="D40" s="135"/>
-      <c r="E40" s="64"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="143"/>
-      <c r="H40" s="143"/>
-      <c r="I40" s="53"/>
-      <c r="J40" s="53"/>
-      <c r="K40" s="53"/>
-      <c r="L40" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="17"/>
-      <c r="B41" s="135" t="s">
-        <v>50</v>
-      </c>
-      <c r="C41" s="135"/>
-      <c r="D41" s="135"/>
-      <c r="E41" s="70"/>
-      <c r="F41" s="19"/>
-      <c r="G41" s="143"/>
-      <c r="H41" s="143"/>
-      <c r="I41" s="53"/>
-      <c r="J41" s="53"/>
-      <c r="K41" s="53"/>
-      <c r="L41" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="17"/>
-      <c r="B42" s="145"/>
-      <c r="C42" s="145"/>
-      <c r="D42" s="145"/>
-      <c r="E42" s="88"/>
-      <c r="F42" s="19"/>
-      <c r="G42" s="108"/>
-      <c r="H42" s="108"/>
-      <c r="I42" s="53"/>
-      <c r="J42" s="53"/>
-      <c r="K42" s="53"/>
-      <c r="L42" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="17"/>
-      <c r="B43" s="117" t="s">
-        <v>51</v>
-      </c>
-      <c r="C43" s="117"/>
-      <c r="D43" s="117"/>
-      <c r="E43" s="117"/>
-      <c r="F43" s="19"/>
-      <c r="G43" s="108"/>
-      <c r="H43" s="108"/>
-      <c r="I43" s="53"/>
-      <c r="J43" s="53"/>
-      <c r="K43" s="53"/>
-      <c r="L43" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="17"/>
-      <c r="B44" s="135" t="s">
-        <v>51</v>
-      </c>
-      <c r="C44" s="135"/>
-      <c r="D44" s="135"/>
-      <c r="E44" s="87" t="s">
-        <v>52</v>
-      </c>
-      <c r="F44" s="19"/>
-      <c r="G44" s="108"/>
-      <c r="H44" s="108"/>
-      <c r="I44" s="53"/>
-      <c r="J44" s="53"/>
-      <c r="K44" s="53"/>
-      <c r="L44" s="49" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="17"/>
-      <c r="B45" s="135" t="s">
-        <v>53</v>
-      </c>
-      <c r="C45" s="135"/>
-      <c r="D45" s="135"/>
-      <c r="E45" s="70"/>
-      <c r="F45" s="19"/>
-      <c r="G45" s="110"/>
-      <c r="H45" s="110"/>
-      <c r="I45" s="56"/>
-      <c r="J45" s="56"/>
-      <c r="K45" s="56"/>
-      <c r="L45" s="57" t="str">
-        <f t="shared" si="0"/>
-        <v>0 H</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="17"/>
-      <c r="B46" s="135" t="s">
-        <v>54</v>
-      </c>
-      <c r="C46" s="135"/>
-      <c r="D46" s="135"/>
-      <c r="E46" s="58"/>
-      <c r="F46" s="19"/>
-      <c r="G46" s="136" t="s">
-        <v>34</v>
-      </c>
-      <c r="H46" s="136"/>
-      <c r="I46" s="74">
-        <f>SUM(I28:I45)</f>
-        <v>550</v>
-      </c>
-      <c r="J46" s="74">
-        <f>SUM(J28:J45)</f>
-        <v>150</v>
-      </c>
-      <c r="K46" s="74">
-        <f>SUM(K28:K45)</f>
-        <v>0</v>
-      </c>
-      <c r="L46" s="72" t="str">
-        <f>J46/50&amp;" HEURES"</f>
-        <v>3 HEURES</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="17"/>
-      <c r="B47" s="111"/>
-      <c r="C47" s="111"/>
-      <c r="D47" s="111"/>
-      <c r="E47" s="111"/>
-      <c r="F47" s="19"/>
-      <c r="G47" s="19"/>
-      <c r="H47" s="19"/>
-      <c r="I47" s="19"/>
-      <c r="J47" s="19"/>
-      <c r="K47" s="19"/>
-      <c r="L47" s="19"/>
-    </row>
-    <row r="48" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="17"/>
-      <c r="B48" s="146" t="s">
-        <v>55</v>
-      </c>
-      <c r="C48" s="146"/>
-      <c r="D48" s="146"/>
-      <c r="E48" s="146"/>
-      <c r="F48" s="146"/>
-      <c r="G48" s="146"/>
-      <c r="H48" s="146"/>
-      <c r="I48" s="146"/>
-      <c r="J48" s="146"/>
-      <c r="K48" s="146"/>
-      <c r="L48" s="146"/>
-    </row>
-    <row r="49" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="17"/>
-      <c r="B49" s="147" t="s">
-        <v>58</v>
-      </c>
-      <c r="C49" s="147"/>
-      <c r="D49" s="147"/>
-      <c r="E49" s="147"/>
-      <c r="F49" s="147"/>
-      <c r="G49" s="147"/>
-      <c r="H49" s="147"/>
-      <c r="I49" s="147"/>
-      <c r="J49" s="147"/>
-      <c r="K49" s="147"/>
-      <c r="L49" s="147"/>
-    </row>
-    <row r="50" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="17"/>
-      <c r="B50" s="114"/>
-      <c r="C50" s="114"/>
-      <c r="D50" s="114"/>
-      <c r="E50" s="114"/>
-      <c r="F50" s="114"/>
-      <c r="G50" s="114"/>
-      <c r="H50" s="114"/>
-      <c r="I50" s="114"/>
-      <c r="J50" s="114"/>
-      <c r="K50" s="114"/>
-      <c r="L50" s="114"/>
-    </row>
-    <row r="51" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="17"/>
-      <c r="B51" s="114"/>
-      <c r="C51" s="114"/>
-      <c r="D51" s="114"/>
-      <c r="E51" s="114"/>
-      <c r="F51" s="114"/>
-      <c r="G51" s="114"/>
-      <c r="H51" s="114"/>
-      <c r="I51" s="114"/>
-      <c r="J51" s="114"/>
-      <c r="K51" s="114"/>
-      <c r="L51" s="114"/>
-    </row>
-    <row r="52" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="17"/>
-      <c r="B52" s="114"/>
-      <c r="C52" s="114"/>
-      <c r="D52" s="114"/>
-      <c r="E52" s="114"/>
-      <c r="F52" s="114"/>
-      <c r="G52" s="114"/>
-      <c r="H52" s="114"/>
-      <c r="I52" s="114"/>
-      <c r="J52" s="114"/>
-      <c r="K52" s="114"/>
-      <c r="L52" s="114"/>
-    </row>
-    <row r="53" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="17"/>
-      <c r="B53" s="114"/>
-      <c r="C53" s="114"/>
-      <c r="D53" s="114"/>
-      <c r="E53" s="114"/>
-      <c r="F53" s="114"/>
-      <c r="G53" s="114"/>
-      <c r="H53" s="114"/>
-      <c r="I53" s="114"/>
-      <c r="J53" s="114"/>
-      <c r="K53" s="114"/>
-      <c r="L53" s="114"/>
-    </row>
-    <row r="54" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="17"/>
-      <c r="B54" s="114"/>
-      <c r="C54" s="114"/>
-      <c r="D54" s="114"/>
-      <c r="E54" s="114"/>
-      <c r="F54" s="114"/>
-      <c r="G54" s="114"/>
-      <c r="H54" s="114"/>
-      <c r="I54" s="114"/>
-      <c r="J54" s="114"/>
-      <c r="K54" s="114"/>
-      <c r="L54" s="114"/>
-    </row>
-    <row r="55" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="17"/>
-      <c r="B55" s="114"/>
-      <c r="C55" s="114"/>
-      <c r="D55" s="114"/>
-      <c r="E55" s="114"/>
-      <c r="F55" s="114"/>
-      <c r="G55" s="114"/>
-      <c r="H55" s="114"/>
-      <c r="I55" s="114"/>
-      <c r="J55" s="114"/>
-      <c r="K55" s="114"/>
-      <c r="L55" s="114"/>
-    </row>
-    <row r="56" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="17"/>
-      <c r="B56" s="114"/>
-      <c r="C56" s="114"/>
-      <c r="D56" s="114"/>
-      <c r="E56" s="114"/>
-      <c r="F56" s="114"/>
-      <c r="G56" s="114"/>
-      <c r="H56" s="114"/>
-      <c r="I56" s="114"/>
-      <c r="J56" s="114"/>
-      <c r="K56" s="114"/>
-      <c r="L56" s="114"/>
-    </row>
-    <row r="57" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="17"/>
-      <c r="B57" s="114"/>
-      <c r="C57" s="114"/>
-      <c r="D57" s="114"/>
-      <c r="E57" s="114"/>
-      <c r="F57" s="114"/>
-      <c r="G57" s="114"/>
-      <c r="H57" s="114"/>
-      <c r="I57" s="114"/>
-      <c r="J57" s="114"/>
-      <c r="K57" s="114"/>
-      <c r="L57" s="114"/>
-    </row>
-    <row r="58" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="17"/>
-      <c r="B58" s="147" t="s">
-        <v>57</v>
-      </c>
-      <c r="C58" s="147"/>
-      <c r="D58" s="147"/>
-      <c r="E58" s="147"/>
-      <c r="F58" s="147"/>
-      <c r="G58" s="147"/>
-      <c r="H58" s="147"/>
-      <c r="I58" s="147"/>
-      <c r="J58" s="147"/>
-      <c r="K58" s="147"/>
-      <c r="L58" s="147"/>
-    </row>
-    <row r="59" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="17"/>
-      <c r="B59" s="114"/>
-      <c r="C59" s="114"/>
-      <c r="D59" s="114"/>
-      <c r="E59" s="114"/>
-      <c r="F59" s="114"/>
-      <c r="G59" s="114"/>
-      <c r="H59" s="114"/>
-      <c r="I59" s="114"/>
-      <c r="J59" s="114"/>
-      <c r="K59" s="114"/>
-      <c r="L59" s="114"/>
-    </row>
-    <row r="60" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="17"/>
-      <c r="B60" s="114"/>
-      <c r="C60" s="114"/>
-      <c r="D60" s="114"/>
-      <c r="E60" s="114"/>
-      <c r="F60" s="114"/>
-      <c r="G60" s="114"/>
-      <c r="H60" s="114"/>
-      <c r="I60" s="114"/>
-      <c r="J60" s="114"/>
-      <c r="K60" s="114"/>
-      <c r="L60" s="114"/>
-    </row>
-    <row r="61" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="17"/>
-      <c r="B61" s="114"/>
-      <c r="C61" s="114"/>
-      <c r="D61" s="114"/>
-      <c r="E61" s="114"/>
-      <c r="F61" s="114"/>
-      <c r="G61" s="114"/>
-      <c r="H61" s="114"/>
-      <c r="I61" s="114"/>
-      <c r="J61" s="114"/>
-      <c r="K61" s="114"/>
-      <c r="L61" s="114"/>
-    </row>
-    <row r="62" spans="1:12" s="15" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="17"/>
-      <c r="B62" s="114"/>
-      <c r="C62" s="114"/>
-      <c r="D62" s="114"/>
-      <c r="E62" s="114"/>
-      <c r="F62" s="114"/>
-      <c r="G62" s="114"/>
-      <c r="H62" s="114"/>
-      <c r="I62" s="114"/>
-      <c r="J62" s="114"/>
-      <c r="K62" s="114"/>
-      <c r="L62" s="114"/>
-    </row>
-    <row r="63" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="17"/>
-      <c r="B63" s="114"/>
-      <c r="C63" s="114"/>
-      <c r="D63" s="114"/>
-      <c r="E63" s="114"/>
-      <c r="F63" s="114"/>
-      <c r="G63" s="114"/>
-      <c r="H63" s="114"/>
-      <c r="I63" s="114"/>
-      <c r="J63" s="114"/>
-      <c r="K63" s="114"/>
-      <c r="L63" s="114"/>
-    </row>
-    <row r="64" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="17"/>
-      <c r="B64" s="147" t="s">
-        <v>56</v>
-      </c>
-      <c r="C64" s="147"/>
-      <c r="D64" s="147"/>
-      <c r="E64" s="147"/>
-      <c r="F64" s="147"/>
-      <c r="G64" s="147"/>
-      <c r="H64" s="147"/>
-      <c r="I64" s="147"/>
-      <c r="J64" s="147"/>
-      <c r="K64" s="147"/>
-      <c r="L64" s="147"/>
-    </row>
-    <row r="65" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="17"/>
-      <c r="B65" s="114"/>
-      <c r="C65" s="114"/>
-      <c r="D65" s="114"/>
-      <c r="E65" s="114"/>
-      <c r="F65" s="114"/>
-      <c r="G65" s="114"/>
-      <c r="H65" s="114"/>
-      <c r="I65" s="114"/>
-      <c r="J65" s="114"/>
-      <c r="K65" s="114"/>
-      <c r="L65" s="114"/>
-    </row>
-    <row r="66" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="17"/>
-      <c r="B66" s="114"/>
-      <c r="C66" s="114"/>
-      <c r="D66" s="114"/>
-      <c r="E66" s="114"/>
-      <c r="F66" s="114"/>
-      <c r="G66" s="114"/>
-      <c r="H66" s="114"/>
-      <c r="I66" s="114"/>
-      <c r="J66" s="114"/>
-      <c r="K66" s="114"/>
-      <c r="L66" s="114"/>
-    </row>
-    <row r="67" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="17"/>
-      <c r="B67" s="114"/>
-      <c r="C67" s="114"/>
-      <c r="D67" s="114"/>
-      <c r="E67" s="114"/>
-      <c r="F67" s="114"/>
-      <c r="G67" s="114"/>
-      <c r="H67" s="114"/>
-      <c r="I67" s="114"/>
-      <c r="J67" s="114"/>
-      <c r="K67" s="114"/>
-      <c r="L67" s="114"/>
-    </row>
-    <row r="68" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="17"/>
-      <c r="B68" s="114"/>
-      <c r="C68" s="114"/>
-      <c r="D68" s="114"/>
-      <c r="E68" s="114"/>
-      <c r="F68" s="114"/>
-      <c r="G68" s="114"/>
-      <c r="H68" s="114"/>
-      <c r="I68" s="114"/>
-      <c r="J68" s="114"/>
-      <c r="K68" s="114"/>
-      <c r="L68" s="114"/>
-    </row>
-    <row r="69" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="17"/>
-      <c r="B69" s="114"/>
-      <c r="C69" s="114"/>
-      <c r="D69" s="114"/>
-      <c r="E69" s="114"/>
-      <c r="F69" s="114"/>
-      <c r="G69" s="114"/>
-      <c r="H69" s="114"/>
-      <c r="I69" s="114"/>
-      <c r="J69" s="114"/>
-      <c r="K69" s="114"/>
-      <c r="L69" s="114"/>
-    </row>
-    <row r="70" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="17"/>
-      <c r="B70" s="117" t="s">
-        <v>59</v>
-      </c>
-      <c r="C70" s="117"/>
-      <c r="D70" s="117"/>
-      <c r="E70" s="117"/>
-      <c r="F70" s="117"/>
-      <c r="G70" s="117"/>
-      <c r="H70" s="117"/>
-      <c r="I70" s="117"/>
-      <c r="J70" s="117"/>
-      <c r="K70" s="117"/>
-      <c r="L70" s="117"/>
-    </row>
-    <row r="71" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="17"/>
-      <c r="B71" s="136" t="s">
-        <v>60</v>
-      </c>
-      <c r="C71" s="136"/>
-      <c r="D71" s="136"/>
-      <c r="E71" s="136"/>
-      <c r="F71" s="136"/>
-      <c r="G71" s="75" t="s">
-        <v>61</v>
-      </c>
-      <c r="H71" s="75" t="s">
-        <v>62</v>
-      </c>
-      <c r="I71" s="75" t="s">
-        <v>63</v>
-      </c>
-      <c r="J71" s="75" t="s">
-        <v>64</v>
-      </c>
-      <c r="K71" s="139" t="s">
-        <v>65</v>
-      </c>
-      <c r="L71" s="139"/>
-    </row>
-    <row r="72" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="17"/>
-      <c r="B72" s="124"/>
-      <c r="C72" s="124"/>
-      <c r="D72" s="124"/>
-      <c r="E72" s="124"/>
-      <c r="F72" s="124"/>
-      <c r="G72" s="89"/>
-      <c r="H72" s="90"/>
-      <c r="I72" s="90"/>
-      <c r="J72" s="90"/>
-      <c r="K72" s="124"/>
-      <c r="L72" s="124"/>
-    </row>
-    <row r="73" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="17"/>
-      <c r="B73" s="124"/>
-      <c r="C73" s="124"/>
-      <c r="D73" s="124"/>
-      <c r="E73" s="124"/>
-      <c r="F73" s="124"/>
-      <c r="G73" s="89"/>
-      <c r="H73" s="90"/>
-      <c r="I73" s="90"/>
-      <c r="J73" s="90"/>
-      <c r="K73" s="124"/>
-      <c r="L73" s="124"/>
-    </row>
-    <row r="74" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="17"/>
-      <c r="B74" s="124"/>
-      <c r="C74" s="124"/>
-      <c r="D74" s="124"/>
-      <c r="E74" s="124"/>
-      <c r="F74" s="124"/>
-      <c r="G74" s="89"/>
-      <c r="H74" s="90"/>
-      <c r="I74" s="90"/>
-      <c r="J74" s="90"/>
-      <c r="K74" s="124"/>
-      <c r="L74" s="124"/>
-    </row>
-    <row r="75" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="17"/>
-      <c r="B75" s="124"/>
-      <c r="C75" s="124"/>
-      <c r="D75" s="124"/>
-      <c r="E75" s="124"/>
-      <c r="F75" s="124"/>
-      <c r="G75" s="89"/>
-      <c r="H75" s="90"/>
-      <c r="I75" s="90"/>
-      <c r="J75" s="90"/>
-      <c r="K75" s="124"/>
-      <c r="L75" s="124"/>
-    </row>
-    <row r="76" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="17"/>
-      <c r="B76" s="124"/>
-      <c r="C76" s="124"/>
-      <c r="D76" s="124"/>
-      <c r="E76" s="124"/>
-      <c r="F76" s="124"/>
-      <c r="G76" s="89"/>
-      <c r="H76" s="90"/>
-      <c r="I76" s="90"/>
-      <c r="J76" s="90"/>
-      <c r="K76" s="124"/>
-      <c r="L76" s="124"/>
-    </row>
-    <row r="77" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="17"/>
-      <c r="B77" s="124"/>
-      <c r="C77" s="124"/>
-      <c r="D77" s="124"/>
-      <c r="E77" s="124"/>
-      <c r="F77" s="124"/>
-      <c r="G77" s="89"/>
-      <c r="H77" s="90"/>
-      <c r="I77" s="90"/>
-      <c r="J77" s="90"/>
-      <c r="K77" s="124"/>
-      <c r="L77" s="124"/>
-    </row>
-    <row r="78" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B78" s="124"/>
-      <c r="C78" s="124"/>
-      <c r="D78" s="124"/>
-      <c r="E78" s="124"/>
-      <c r="F78" s="124"/>
-      <c r="G78" s="89"/>
-      <c r="H78" s="90"/>
-      <c r="I78" s="90"/>
-      <c r="J78" s="90"/>
-      <c r="K78" s="124"/>
-      <c r="L78" s="124"/>
-    </row>
-    <row r="79" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B79" s="124"/>
-      <c r="C79" s="124"/>
-      <c r="D79" s="124"/>
-      <c r="E79" s="124"/>
-      <c r="F79" s="124"/>
-      <c r="G79" s="89"/>
-      <c r="H79" s="90"/>
-      <c r="I79" s="90"/>
-      <c r="J79" s="90"/>
-      <c r="K79" s="124"/>
-      <c r="L79" s="124"/>
-    </row>
-    <row r="80" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B80" s="124"/>
-      <c r="C80" s="124"/>
-      <c r="D80" s="124"/>
-      <c r="E80" s="124"/>
-      <c r="F80" s="124"/>
-      <c r="G80" s="89"/>
-      <c r="H80" s="90"/>
-      <c r="I80" s="90"/>
-      <c r="J80" s="90"/>
-      <c r="K80" s="124"/>
-      <c r="L80" s="124"/>
-    </row>
-    <row r="81" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B81" s="62"/>
-      <c r="C81" s="62"/>
-      <c r="D81" s="62"/>
-      <c r="E81" s="62"/>
-      <c r="F81" s="62"/>
-      <c r="G81" s="62"/>
-      <c r="H81" s="62"/>
-      <c r="I81" s="62"/>
-      <c r="J81" s="62"/>
-      <c r="K81" s="62"/>
-      <c r="L81" s="17"/>
-    </row>
-  </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="aSNUIXnI8lIlIiS8Zr0Zm4BOh4G2UpoxzoJn9g4sSDNFsQCXSl57ZB78zeYMNTCfcVjOQHXJiDsPsY2GQDViuA==" saltValue="erzlKi8xbvgTP9ReDVFkaA==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
-  <mergeCells count="143">
-    <mergeCell ref="B77:F77"/>
-    <mergeCell ref="K77:L77"/>
-    <mergeCell ref="B78:F78"/>
-    <mergeCell ref="K78:L78"/>
-    <mergeCell ref="B79:F79"/>
-    <mergeCell ref="K79:L79"/>
-    <mergeCell ref="B80:F80"/>
-    <mergeCell ref="K80:L80"/>
-    <mergeCell ref="B72:F72"/>
-    <mergeCell ref="K72:L72"/>
-    <mergeCell ref="B73:F73"/>
-    <mergeCell ref="K73:L73"/>
-    <mergeCell ref="B74:F74"/>
-    <mergeCell ref="K74:L74"/>
-    <mergeCell ref="B75:F75"/>
-    <mergeCell ref="K75:L75"/>
-    <mergeCell ref="B76:F76"/>
-    <mergeCell ref="K76:L76"/>
-    <mergeCell ref="B63:L63"/>
-    <mergeCell ref="B64:L64"/>
-    <mergeCell ref="B65:L65"/>
-    <mergeCell ref="B66:L66"/>
-    <mergeCell ref="B67:L67"/>
-    <mergeCell ref="B68:L68"/>
-    <mergeCell ref="B69:L69"/>
-    <mergeCell ref="B70:L70"/>
-    <mergeCell ref="B71:F71"/>
-    <mergeCell ref="K71:L71"/>
-    <mergeCell ref="B54:L54"/>
-    <mergeCell ref="B55:L55"/>
-    <mergeCell ref="B56:L56"/>
-    <mergeCell ref="B57:L57"/>
-    <mergeCell ref="B58:L58"/>
-    <mergeCell ref="B59:L59"/>
-    <mergeCell ref="B60:L60"/>
-    <mergeCell ref="B61:L61"/>
-    <mergeCell ref="B62:L62"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="B48:L48"/>
-    <mergeCell ref="B49:L49"/>
-    <mergeCell ref="B50:L50"/>
-    <mergeCell ref="B51:L51"/>
-    <mergeCell ref="B52:L52"/>
-    <mergeCell ref="B53:L53"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="B43:E43"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="G33:H33"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="G26:L26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="G11:L11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="K12:L12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="K13:L13"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="I7:L7"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="G8:H9"/>
-    <mergeCell ref="I8:J9"/>
-    <mergeCell ref="K8:L9"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="G10:K10"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:L4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="G5:H6"/>
-    <mergeCell ref="I5:J6"/>
-    <mergeCell ref="K5:L6"/>
-    <mergeCell ref="C6:E6"/>
-  </mergeCells>
-  <conditionalFormatting sqref="B34:E34">
-    <cfRule type="expression" dxfId="4" priority="2">
-      <formula>$E$34&gt;$E$30</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
-      <formula>$E$34&gt;$E$30</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4">
-      <formula>$E$34&gt;$E$30</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="5" operator="greaterThan">
-      <formula>$E$34&gt;$E$30</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="6">
-      <formula>$E$34&gt;$E$30</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="7">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E39 E44" xr:uid="{00000000-0002-0000-0100-000000000000}">
-      <formula1>OUINON</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J13:J16 J18 J20:J23" xr:uid="{00000000-0002-0000-0100-000001000000}">
-      <formula1>"OUI,NON"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J17 J19" xr:uid="{00000000-0002-0000-0100-000002000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E40" xr:uid="{00000000-0002-0000-0100-000004000000}">
-      <formula1>"CETELEM,FINANCO,LOISIRS FI,SANTANDER,VIAXEL"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G8:H9" xr:uid="{00000000-0002-0000-0100-000005000000}">
-      <formula1>"Moins de 360 jours,Entre 361 et 700 jours,Plus de 701 jours"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G29:H29" xr:uid="{00000000-0002-0000-0100-000006000000}">
-      <formula1>"Préparation esthétique par sous-traitant,Préparation déjà réalisée,Pas de préparation esthétique"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5:H6" xr:uid="{00000000-0002-0000-0100-000007000000}">
-      <formula1>"CAMPING CAR,CARAVANE,PROTO A MARCHAND (VDL &gt; 2014),PROTO A MARCHAND (VDL &lt; 2014)"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
-  <printOptions horizontalCentered="1" verticalCentered="1"/>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.31527777777777799"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
-  <headerFooter>
-    <oddFooter>&amp;L&amp;F&amp;CRENTA VN&amp;R&amp;D &amp;T</oddFooter>
-  </headerFooter>
-  <legacyDrawing r:id="rId1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A3:B5"/>

</xml_diff>

<commit_message>
REF ODOO sans décimale
</commit_message>
<xml_diff>
--- a/public/templates/trame_renta_template.xlsx
+++ b/public/templates/trame_renta_template.xlsx
@@ -1010,7 +1010,7 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="149">
+  <cellXfs count="150">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1489,6 +1489,9 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1993,7 +1996,7 @@
       <c r="B8" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="149">
         <f>IF(E35=0,(E34*9%),(E34*11%+E40*0.3%))</f>
         <v>0</v>
       </c>

</xml_diff>